<commit_message>
Lohnabrechnung-PDF: 'EVENTLINE GmbH' Text weg (Logo steht's drauf)
</commit_message>
<xml_diff>
--- a/examples/timesheet_sample.xlsx
+++ b/examples/timesheet_sample.xlsx
@@ -227,19 +227,19 @@
     <t>Brutto-Lohnkosten</t>
   </si>
   <si>
-    <t>CHF 7'267.03</t>
+    <t>CHF 7'280.80</t>
   </si>
   <si>
     <t>Netto-Auszahlung</t>
   </si>
   <si>
-    <t>CHF 6'700.20</t>
+    <t>CHF 6'712.90</t>
   </si>
   <si>
     <t>Vollkosten Arbeitgeber</t>
   </si>
   <si>
-    <t>CHF 8'026.66</t>
+    <t>CHF 8'042.08</t>
   </si>
   <si>
     <t>Hinweis</t>
@@ -269,13 +269,13 @@
     <t>CHF 32.31 / h</t>
   </si>
   <si>
-    <t>CHF 8'464.75</t>
-  </si>
-  <si>
-    <t>CHF 7'804.50</t>
-  </si>
-  <si>
-    <t>CHF 9'326.28</t>
+    <t>CHF 8'426.25</t>
+  </si>
+  <si>
+    <t>CHF 7'769.00</t>
+  </si>
+  <si>
+    <t>CHF 9'283.20</t>
   </si>
   <si>
     <t>2026-03-07</t>
@@ -299,13 +299,13 @@
     <t>CHF 16.45 / h</t>
   </si>
   <si>
-    <t>CHF 4'851.51</t>
-  </si>
-  <si>
-    <t>CHF 4'473.10</t>
-  </si>
-  <si>
-    <t>CHF 5'376.86</t>
+    <t>CHF 4'849.39</t>
+  </si>
+  <si>
+    <t>CHF 4'471.14</t>
+  </si>
+  <si>
+    <t>CHF 5'374.49</t>
   </si>
   <si>
     <t>Zeitraum</t>
@@ -960,10 +960,10 @@
         <v>224</v>
       </c>
       <c r="D2">
-        <v>142</v>
+        <v>170</v>
       </c>
       <c r="E2">
-        <v>223.98</v>
+        <v>224.47</v>
       </c>
       <c r="F2">
         <v>44</v>
@@ -972,13 +972,13 @@
         <v>4</v>
       </c>
       <c r="H2">
-        <v>7267.02</v>
+        <v>7280.8</v>
       </c>
       <c r="I2">
-        <v>6700.2</v>
+        <v>6712.9</v>
       </c>
       <c r="J2">
-        <v>8026.66</v>
+        <v>8042.08</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -992,10 +992,10 @@
         <v>206</v>
       </c>
       <c r="D3">
-        <v>144</v>
+        <v>190</v>
       </c>
       <c r="E3">
-        <v>206.85</v>
+        <v>205.75</v>
       </c>
       <c r="F3">
         <v>44</v>
@@ -1004,13 +1004,13 @@
         <v>5</v>
       </c>
       <c r="H3">
-        <v>8464.75</v>
+        <v>8426.25</v>
       </c>
       <c r="I3">
-        <v>7804.5</v>
+        <v>7769</v>
       </c>
       <c r="J3">
-        <v>9326.28</v>
+        <v>9283.2</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -1027,7 +1027,7 @@
         <v>204</v>
       </c>
       <c r="E4">
-        <v>242.57</v>
+        <v>242.45</v>
       </c>
       <c r="F4">
         <v>44</v>
@@ -1036,13 +1036,13 @@
         <v>3</v>
       </c>
       <c r="H4">
-        <v>4851.51</v>
+        <v>4849.39</v>
       </c>
       <c r="I4">
-        <v>4473.1</v>
+        <v>4471.14</v>
       </c>
       <c r="J4">
-        <v>5376.86</v>
+        <v>5374.49</v>
       </c>
     </row>
   </sheetData>
@@ -1115,7 +1115,7 @@
         <v>600</v>
       </c>
       <c r="G2">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="H2">
         <v>10</v>
@@ -1144,7 +1144,7 @@
         <v>600</v>
       </c>
       <c r="G3">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="H3">
         <v>10</v>
@@ -1170,10 +1170,10 @@
         <v>300</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="G4">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="H4">
         <v>8</v>
@@ -1202,7 +1202,7 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="H5">
         <v>10</v>
@@ -1231,7 +1231,7 @@
         <v>600</v>
       </c>
       <c r="G6">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="H6">
         <v>10</v>
@@ -1260,7 +1260,7 @@
         <v>600</v>
       </c>
       <c r="G7">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H7">
         <v>10</v>
@@ -1289,7 +1289,7 @@
         <v>600</v>
       </c>
       <c r="G8">
-        <v>606</v>
+        <v>599</v>
       </c>
       <c r="H8">
         <v>10</v>
@@ -1318,7 +1318,7 @@
         <v>600</v>
       </c>
       <c r="G9">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="H9">
         <v>10</v>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="H10">
         <v>8</v>
@@ -1376,7 +1376,7 @@
         <v>600</v>
       </c>
       <c r="G11">
-        <v>608</v>
+        <v>602</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -1402,10 +1402,10 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G12">
-        <v>605</v>
+        <v>597</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -1434,7 +1434,7 @@
         <v>480</v>
       </c>
       <c r="G13">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="H13">
         <v>8</v>
@@ -1460,10 +1460,10 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G14">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="H14">
         <v>10</v>
@@ -1492,7 +1492,7 @@
         <v>600</v>
       </c>
       <c r="G15">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="H15">
         <v>10</v>
@@ -1518,10 +1518,10 @@
         <v>0</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="G16">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="H16">
         <v>8</v>
@@ -1550,7 +1550,7 @@
         <v>600</v>
       </c>
       <c r="G17">
-        <v>602</v>
+        <v>614</v>
       </c>
       <c r="H17">
         <v>10</v>
@@ -1576,7 +1576,7 @@
         <v>0</v>
       </c>
       <c r="F18">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G18">
         <v>614</v>
@@ -1634,10 +1634,10 @@
         <v>0</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="G20">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="H20">
         <v>8</v>
@@ -1663,10 +1663,10 @@
         <v>180</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G21">
-        <v>587</v>
+        <v>611</v>
       </c>
       <c r="H21">
         <v>10</v>
@@ -1695,7 +1695,7 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="H22">
         <v>10</v>
@@ -1721,10 +1721,10 @@
         <v>300</v>
       </c>
       <c r="F23">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="H23">
         <v>8</v>
@@ -1753,7 +1753,7 @@
         <v>600</v>
       </c>
       <c r="G24">
-        <v>594</v>
+        <v>588</v>
       </c>
       <c r="H24">
         <v>10</v>
@@ -1779,10 +1779,10 @@
         <v>0</v>
       </c>
       <c r="F25">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>489</v>
+        <v>469</v>
       </c>
       <c r="H25">
         <v>8</v>
@@ -1802,10 +1802,10 @@
         <v>2640</v>
       </c>
       <c r="F26" s="2">
-        <v>8520</v>
+        <v>10200</v>
       </c>
       <c r="G26" s="2">
-        <v>13439</v>
+        <v>13468</v>
       </c>
       <c r="H26" s="2">
         <v>224</v>
@@ -1845,7 +1845,7 @@
         <v>66</v>
       </c>
       <c r="I32">
-        <v>13439</v>
+        <v>13468</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -1853,7 +1853,7 @@
         <v>67</v>
       </c>
       <c r="I33">
-        <v>13439</v>
+        <v>13468</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -1966,7 +1966,7 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="H2">
         <v>8</v>
@@ -1995,7 +1995,7 @@
         <v>480</v>
       </c>
       <c r="G3">
-        <v>472</v>
+        <v>483</v>
       </c>
       <c r="H3">
         <v>8</v>
@@ -2024,7 +2024,7 @@
         <v>600</v>
       </c>
       <c r="G4">
-        <v>610</v>
+        <v>590</v>
       </c>
       <c r="H4">
         <v>10</v>
@@ -2050,10 +2050,10 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G5">
-        <v>592</v>
+        <v>610</v>
       </c>
       <c r="H5">
         <v>10</v>
@@ -2079,10 +2079,10 @@
         <v>300</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="G6">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H6">
         <v>8</v>
@@ -2111,7 +2111,7 @@
         <v>600</v>
       </c>
       <c r="G7">
-        <v>613</v>
+        <v>596</v>
       </c>
       <c r="H7">
         <v>10</v>
@@ -2137,10 +2137,10 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="G8">
-        <v>495</v>
+        <v>466</v>
       </c>
       <c r="H8">
         <v>8</v>
@@ -2166,7 +2166,7 @@
         <v>180</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G9">
         <v>603</v>
@@ -2198,7 +2198,7 @@
         <v>600</v>
       </c>
       <c r="G10">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="H10">
         <v>10</v>
@@ -2227,7 +2227,7 @@
         <v>480</v>
       </c>
       <c r="G11">
-        <v>493</v>
+        <v>477</v>
       </c>
       <c r="H11">
         <v>8</v>
@@ -2256,7 +2256,7 @@
         <v>600</v>
       </c>
       <c r="G12">
-        <v>613</v>
+        <v>585</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -2285,7 +2285,7 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>476</v>
+        <v>486</v>
       </c>
       <c r="H13">
         <v>8</v>
@@ -2314,7 +2314,7 @@
         <v>600</v>
       </c>
       <c r="G14">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="H14">
         <v>10</v>
@@ -2343,7 +2343,7 @@
         <v>600</v>
       </c>
       <c r="G15">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="H15">
         <v>10</v>
@@ -2372,7 +2372,7 @@
         <v>600</v>
       </c>
       <c r="G16">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="H16">
         <v>10</v>
@@ -2401,7 +2401,7 @@
         <v>600</v>
       </c>
       <c r="G17">
-        <v>612</v>
+        <v>596</v>
       </c>
       <c r="H17">
         <v>10</v>
@@ -2430,7 +2430,7 @@
         <v>600</v>
       </c>
       <c r="G18">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="H18">
         <v>10</v>
@@ -2459,7 +2459,7 @@
         <v>480</v>
       </c>
       <c r="G19">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="H19">
         <v>8</v>
@@ -2488,7 +2488,7 @@
         <v>600</v>
       </c>
       <c r="G20">
-        <v>604</v>
+        <v>594</v>
       </c>
       <c r="H20">
         <v>10</v>
@@ -2517,7 +2517,7 @@
         <v>600</v>
       </c>
       <c r="G21">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="H21">
         <v>10</v>
@@ -2546,7 +2546,7 @@
         <v>600</v>
       </c>
       <c r="G22">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="H22">
         <v>10</v>
@@ -2572,10 +2572,10 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G23">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="H23">
         <v>10</v>
@@ -2595,10 +2595,10 @@
         <v>2640</v>
       </c>
       <c r="F24" s="2">
-        <v>8640</v>
+        <v>11400</v>
       </c>
       <c r="G24" s="2">
-        <v>12411</v>
+        <v>12345</v>
       </c>
       <c r="H24" s="2">
         <v>206</v>
@@ -2638,7 +2638,7 @@
         <v>66</v>
       </c>
       <c r="I30">
-        <v>12411</v>
+        <v>12345</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -2646,7 +2646,7 @@
         <v>67</v>
       </c>
       <c r="I31">
-        <v>12411</v>
+        <v>12345</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -2759,7 +2759,7 @@
         <v>600</v>
       </c>
       <c r="G2">
-        <v>606</v>
+        <v>597</v>
       </c>
       <c r="H2">
         <v>10</v>
@@ -2788,7 +2788,7 @@
         <v>480</v>
       </c>
       <c r="G3">
-        <v>494</v>
+        <v>470</v>
       </c>
       <c r="H3">
         <v>8</v>
@@ -2817,7 +2817,7 @@
         <v>600</v>
       </c>
       <c r="G4">
-        <v>601</v>
+        <v>594</v>
       </c>
       <c r="H4">
         <v>10</v>
@@ -2846,7 +2846,7 @@
         <v>600</v>
       </c>
       <c r="G5">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="H5">
         <v>10</v>
@@ -2875,7 +2875,7 @@
         <v>480</v>
       </c>
       <c r="G6">
-        <v>473</v>
+        <v>495</v>
       </c>
       <c r="H6">
         <v>8</v>
@@ -2901,10 +2901,10 @@
         <v>180</v>
       </c>
       <c r="F7">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>597</v>
+        <v>615</v>
       </c>
       <c r="H7">
         <v>10</v>
@@ -2933,7 +2933,7 @@
         <v>600</v>
       </c>
       <c r="G8">
-        <v>605</v>
+        <v>592</v>
       </c>
       <c r="H8">
         <v>10</v>
@@ -2959,10 +2959,10 @@
         <v>300</v>
       </c>
       <c r="F9">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>474</v>
+        <v>489</v>
       </c>
       <c r="H9">
         <v>8</v>
@@ -2988,10 +2988,10 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="G10">
-        <v>478</v>
+        <v>467</v>
       </c>
       <c r="H10">
         <v>8</v>
@@ -3020,7 +3020,7 @@
         <v>600</v>
       </c>
       <c r="G11">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -3049,7 +3049,7 @@
         <v>600</v>
       </c>
       <c r="G12">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -3078,7 +3078,7 @@
         <v>480</v>
       </c>
       <c r="G13">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="H13">
         <v>8</v>
@@ -3107,7 +3107,7 @@
         <v>600</v>
       </c>
       <c r="G14">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="H14">
         <v>10</v>
@@ -3133,10 +3133,10 @@
         <v>180</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G15">
-        <v>612</v>
+        <v>599</v>
       </c>
       <c r="H15">
         <v>10</v>
@@ -3165,7 +3165,7 @@
         <v>480</v>
       </c>
       <c r="G16">
-        <v>480</v>
+        <v>469</v>
       </c>
       <c r="H16">
         <v>8</v>
@@ -3191,10 +3191,10 @@
         <v>180</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G17">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="H17">
         <v>10</v>
@@ -3220,10 +3220,10 @@
         <v>0</v>
       </c>
       <c r="F18">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="H18">
         <v>10</v>
@@ -3252,7 +3252,7 @@
         <v>480</v>
       </c>
       <c r="G19">
-        <v>471</v>
+        <v>485</v>
       </c>
       <c r="H19">
         <v>8</v>
@@ -3278,10 +3278,10 @@
         <v>0</v>
       </c>
       <c r="F20">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>597</v>
+        <v>612</v>
       </c>
       <c r="H20">
         <v>10</v>
@@ -3310,7 +3310,7 @@
         <v>600</v>
       </c>
       <c r="G21">
-        <v>607</v>
+        <v>599</v>
       </c>
       <c r="H21">
         <v>10</v>
@@ -3339,7 +3339,7 @@
         <v>480</v>
       </c>
       <c r="G22">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="H22">
         <v>8</v>
@@ -3365,10 +3365,10 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G23">
-        <v>607</v>
+        <v>594</v>
       </c>
       <c r="H23">
         <v>10</v>
@@ -3397,7 +3397,7 @@
         <v>600</v>
       </c>
       <c r="G24">
-        <v>603</v>
+        <v>589</v>
       </c>
       <c r="H24">
         <v>10</v>
@@ -3426,7 +3426,7 @@
         <v>600</v>
       </c>
       <c r="G25">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="H25">
         <v>10</v>
@@ -3455,7 +3455,7 @@
         <v>480</v>
       </c>
       <c r="G26">
-        <v>486</v>
+        <v>494</v>
       </c>
       <c r="H26">
         <v>8</v>
@@ -3484,7 +3484,7 @@
         <v>600</v>
       </c>
       <c r="G27">
-        <v>589</v>
+        <v>601</v>
       </c>
       <c r="H27">
         <v>10</v>
@@ -3507,7 +3507,7 @@
         <v>12240</v>
       </c>
       <c r="G28" s="2">
-        <v>14554</v>
+        <v>14547</v>
       </c>
       <c r="H28" s="2">
         <v>242</v>
@@ -3547,7 +3547,7 @@
         <v>66</v>
       </c>
       <c r="I34">
-        <v>14554</v>
+        <v>14547</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -3555,7 +3555,7 @@
         <v>67</v>
       </c>
       <c r="I35">
-        <v>14554</v>
+        <v>14547</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>